<commit_message>
Corrige l'extraction du prix cumulé des challenges
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpnEpdwNF8V8azepdqLgDD
</commit_message>
<xml_diff>
--- a/docs/prop-firms-capital-max.xlsx
+++ b/docs/prop-firms-capital-max.xlsx
@@ -151,10 +151,10 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -969,10 +969,8 @@
       <c r="J3" s="10" t="n">
         <v>2300000</v>
       </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K3" s="10" t="n">
+        <v>6900</v>
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
@@ -1031,7 +1029,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1113,7 +1111,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1196,7 +1194,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1220,10 +1218,8 @@
       <c r="J6" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="K6" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K6" s="10" t="n">
+        <v>3500</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -1305,7 +1301,7 @@
       <c r="J7" s="10" t="n">
         <v>1555000</v>
       </c>
-      <c r="K7" s="13" t="inlineStr">
+      <c r="K7" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -1389,7 +1385,7 @@
       <c r="J8" s="10" t="n">
         <v>1555000</v>
       </c>
-      <c r="K8" s="13" t="inlineStr">
+      <c r="K8" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -1449,7 +1445,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1469,7 +1465,7 @@
       <c r="J9" s="10" t="n">
         <v>1500000</v>
       </c>
-      <c r="K9" s="13" t="inlineStr">
+      <c r="K9" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -1532,7 +1528,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1552,10 +1548,8 @@
       <c r="J10" s="10" t="n">
         <v>1500000</v>
       </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K10" s="10" t="n">
+        <v>23100</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -1615,7 +1609,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1639,7 +1633,7 @@
       <c r="J11" s="10" t="n">
         <v>1250000</v>
       </c>
-      <c r="K11" s="13" t="inlineStr">
+      <c r="K11" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -1720,7 +1714,7 @@
       <c r="J12" s="10" t="n">
         <v>1100000</v>
       </c>
-      <c r="K12" s="13" t="inlineStr">
+      <c r="K12" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -1806,7 +1800,7 @@
       <c r="J13" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K13" s="13" t="inlineStr">
+      <c r="K13" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -1869,7 +1863,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -1889,10 +1883,8 @@
       <c r="J14" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K14" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K14" s="10" t="n">
+        <v>4950</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
@@ -2110,7 +2102,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -2130,10 +2122,8 @@
       <c r="J17" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K17" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K17" s="10" t="n">
+        <v>1622</v>
       </c>
       <c r="L17" s="11" t="inlineStr">
         <is>
@@ -2191,7 +2181,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -2215,7 +2205,7 @@
       <c r="J18" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K18" s="13" t="inlineStr">
+      <c r="K18" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -2299,7 +2289,7 @@
       <c r="J19" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K19" s="13" t="inlineStr">
+      <c r="K19" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -2441,7 +2431,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -2465,10 +2455,8 @@
       <c r="J21" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K21" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K21" s="10" t="n">
+        <v>5040</v>
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
@@ -2525,7 +2513,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -2607,7 +2595,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -2685,7 +2673,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -3032,7 +3020,7 @@
       <c r="J28" s="10" t="n">
         <v>900000</v>
       </c>
-      <c r="K28" s="13" t="inlineStr">
+      <c r="K28" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -3088,12 +3076,12 @@
           <t>CFD + Futures</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -3197,10 +3185,8 @@
       <c r="J30" s="10" t="n">
         <v>800000</v>
       </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K30" s="10" t="n">
+        <v>2398</v>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
@@ -3258,7 +3244,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -3508,7 +3494,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E34" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -3532,7 +3518,7 @@
       <c r="J34" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="K34" s="13" t="inlineStr">
+      <c r="K34" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -3699,10 +3685,8 @@
       <c r="J36" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="K36" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K36" s="10" t="n">
+        <v>1095</v>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
@@ -3759,7 +3743,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E37" s="14" t="inlineStr">
+      <c r="E37" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -3783,10 +3767,8 @@
       <c r="J37" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="K37" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K37" s="10" t="n">
+        <v>2690</v>
       </c>
       <c r="L37" s="11" t="inlineStr">
         <is>
@@ -3867,10 +3849,8 @@
       <c r="J38" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="K38" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K38" s="10" t="n">
+        <v>1600000</v>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
@@ -4115,10 +4095,8 @@
       <c r="J41" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="K41" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K41" s="10" t="n">
+        <v>1490</v>
       </c>
       <c r="L41" s="11" t="inlineStr">
         <is>
@@ -4176,7 +4154,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="E42" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -4200,10 +4178,8 @@
       <c r="J42" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="K42" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K42" s="10" t="n">
+        <v>1800</v>
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
@@ -4261,7 +4237,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E43" s="14" t="inlineStr">
+      <c r="E43" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -4346,7 +4322,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E44" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -4370,10 +4346,8 @@
       <c r="J44" s="10" t="n">
         <v>720000</v>
       </c>
-      <c r="K44" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K44" s="10" t="n">
+        <v>2744</v>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
@@ -4433,7 +4407,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="E45" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -4457,10 +4431,8 @@
       <c r="J45" s="10" t="n">
         <v>700000</v>
       </c>
-      <c r="K45" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K45" s="10" t="n">
+        <v>2818</v>
       </c>
       <c r="L45" s="11" t="inlineStr">
         <is>
@@ -4518,7 +4490,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -4538,7 +4510,7 @@
       <c r="J46" s="10" t="n">
         <v>700000</v>
       </c>
-      <c r="K46" s="13" t="inlineStr">
+      <c r="K46" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -4620,10 +4592,8 @@
       <c r="J47" s="10" t="n">
         <v>640000</v>
       </c>
-      <c r="K47" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K47" s="10" t="n">
+        <v>798</v>
       </c>
       <c r="L47" s="11" t="inlineStr">
         <is>
@@ -4678,12 +4648,12 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr">
+      <c r="D48" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
+      <c r="E48" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -4843,7 +4813,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E50" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -5088,7 +5058,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E53" s="14" t="inlineStr">
+      <c r="E53" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -5112,10 +5082,8 @@
       <c r="J53" s="10" t="n">
         <v>600000</v>
       </c>
-      <c r="K53" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K53" s="10" t="n">
+        <v>2094</v>
       </c>
       <c r="L53" s="11" t="inlineStr">
         <is>
@@ -5249,12 +5217,12 @@
           <t>CFD + Futures</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr">
+      <c r="D55" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E55" s="14" t="inlineStr">
+      <c r="E55" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -5278,10 +5246,8 @@
       <c r="J55" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="K55" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K55" s="10" t="n">
+        <v>1900</v>
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
@@ -5422,7 +5388,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E57" s="14" t="inlineStr">
+      <c r="E57" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -5446,7 +5412,7 @@
       <c r="J57" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="K57" s="13" t="inlineStr">
+      <c r="K57" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -5533,10 +5499,8 @@
       <c r="J58" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="K58" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K58" s="10" t="n">
+        <v>1998</v>
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
@@ -5591,12 +5555,12 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="D59" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E59" s="14" t="inlineStr">
+      <c r="E59" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -5674,7 +5638,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E60" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -5698,10 +5662,8 @@
       <c r="J60" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="K60" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K60" s="10" t="n">
+        <v>2057</v>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
@@ -6022,7 +5984,7 @@
       <c r="J64" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="K64" s="13" t="inlineStr">
+      <c r="K64" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -6085,7 +6047,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E65" s="14" t="inlineStr">
+      <c r="E65" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -6109,7 +6071,7 @@
       <c r="J65" s="10" t="n">
         <v>467500</v>
       </c>
-      <c r="K65" s="13" t="inlineStr">
+      <c r="K65" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -6196,10 +6158,8 @@
       <c r="J66" s="10" t="n">
         <v>450000</v>
       </c>
-      <c r="K66" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K66" s="10" t="n">
+        <v>1362</v>
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
@@ -6257,7 +6217,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E67" s="14" t="inlineStr">
+      <c r="E67" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -6281,10 +6241,8 @@
       <c r="J67" s="10" t="n">
         <v>450000</v>
       </c>
-      <c r="K67" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K67" s="10" t="n">
+        <v>687</v>
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
@@ -6506,7 +6464,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E70" s="14" t="inlineStr">
+      <c r="E70" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -6663,7 +6621,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D72" s="14" t="inlineStr">
+      <c r="D72" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -7073,7 +7031,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E77" s="14" t="inlineStr">
+      <c r="E77" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -7251,10 +7209,8 @@
       <c r="J79" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="K79" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K79" s="10" t="n">
+        <v>1100</v>
       </c>
       <c r="L79" s="11" t="inlineStr">
         <is>
@@ -7476,7 +7432,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E82" s="14" t="inlineStr">
+      <c r="E82" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -7561,7 +7517,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E83" s="14" t="inlineStr">
+      <c r="E83" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -7585,10 +7541,8 @@
       <c r="J83" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="K83" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K83" s="10" t="n">
+        <v>2354</v>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
@@ -7643,12 +7597,12 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D84" s="14" t="inlineStr">
+      <c r="D84" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E84" s="14" t="inlineStr">
+      <c r="E84" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -7731,7 +7685,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E85" s="14" t="inlineStr">
+      <c r="E85" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -7755,10 +7709,8 @@
       <c r="J85" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="K85" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K85" s="10" t="n">
+        <v>899</v>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
@@ -8060,7 +8012,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E89" s="14" t="inlineStr">
+      <c r="E89" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -8137,7 +8089,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D90" s="14" t="inlineStr">
+      <c r="D90" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -8223,7 +8175,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E91" s="14" t="inlineStr">
+      <c r="E91" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -8298,12 +8250,12 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D92" s="14" t="inlineStr">
+      <c r="D92" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E92" s="14" t="inlineStr">
+      <c r="E92" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -8385,7 +8337,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E93" s="14" t="inlineStr">
+      <c r="E93" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -8466,7 +8418,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E94" s="14" t="inlineStr">
+      <c r="E94" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -8567,7 +8519,7 @@
       <c r="J95" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="K95" s="13" t="inlineStr">
+      <c r="K95" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -8733,10 +8685,8 @@
       <c r="J97" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="K97" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K97" s="10" t="n">
+        <v>1777</v>
       </c>
       <c r="L97" s="11" t="inlineStr">
         <is>
@@ -8796,7 +8746,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E98" s="14" t="inlineStr">
+      <c r="E98" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -8816,7 +8766,7 @@
       <c r="J98" s="10" t="n">
         <v>390000</v>
       </c>
-      <c r="K98" s="13" t="inlineStr">
+      <c r="K98" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -8901,10 +8851,8 @@
       <c r="J99" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="K99" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K99" s="10" t="n">
+        <v>1573</v>
       </c>
       <c r="L99" s="11" t="inlineStr">
         <is>
@@ -8982,10 +8930,8 @@
       <c r="J100" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="K100" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K100" s="10" t="n">
+        <v>1399</v>
       </c>
       <c r="L100" s="7" t="inlineStr">
         <is>
@@ -9067,10 +9013,8 @@
       <c r="J101" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="K101" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K101" s="10" t="n">
+        <v>1581</v>
       </c>
       <c r="L101" s="11" t="inlineStr">
         <is>
@@ -9211,7 +9155,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E103" s="14" t="inlineStr">
+      <c r="E103" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -9235,10 +9179,8 @@
       <c r="J103" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="K103" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K103" s="10" t="n">
+        <v>700</v>
       </c>
       <c r="L103" s="11" t="inlineStr">
         <is>
@@ -9377,7 +9319,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E105" s="14" t="inlineStr">
+      <c r="E105" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -9461,7 +9403,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E106" s="14" t="inlineStr">
+      <c r="E106" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -9566,10 +9508,8 @@
       <c r="J107" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="K107" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K107" s="10" t="n">
+        <v>1399</v>
       </c>
       <c r="L107" s="11" t="inlineStr">
         <is>
@@ -9627,7 +9567,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E108" s="14" t="inlineStr">
+      <c r="E108" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -9896,10 +9836,8 @@
       <c r="J111" s="10" t="n">
         <v>250000</v>
       </c>
-      <c r="K111" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K111" s="10" t="n">
+        <v>999</v>
       </c>
       <c r="L111" s="11" t="inlineStr">
         <is>
@@ -9980,7 +9918,7 @@
       <c r="J112" s="10" t="n">
         <v>250000</v>
       </c>
-      <c r="K112" s="13" t="inlineStr">
+      <c r="K112" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -10041,7 +9979,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E113" s="14" t="inlineStr">
+      <c r="E113" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -10065,10 +10003,8 @@
       <c r="J113" s="10" t="n">
         <v>240000</v>
       </c>
-      <c r="K113" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K113" s="10" t="n">
+        <v>5196</v>
       </c>
       <c r="L113" s="11" t="inlineStr">
         <is>
@@ -10152,7 +10088,7 @@
       <c r="J114" s="10" t="n">
         <v>200000</v>
       </c>
-      <c r="K114" s="13" t="inlineStr">
+      <c r="K114" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -10401,10 +10337,8 @@
       <c r="J117" s="10" t="n">
         <v>200000</v>
       </c>
-      <c r="K117" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K117" s="10" t="n">
+        <v>699</v>
       </c>
       <c r="L117" s="11" t="inlineStr">
         <is>
@@ -10547,7 +10481,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E119" s="14" t="inlineStr">
+      <c r="E119" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -10875,7 +10809,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E123" s="14" t="inlineStr">
+      <c r="E123" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -11034,7 +10968,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E125" s="14" t="inlineStr">
+      <c r="E125" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -11143,7 +11077,7 @@
       <c r="J126" s="10" t="n">
         <v>200000</v>
       </c>
-      <c r="K126" s="13" t="inlineStr">
+      <c r="K126" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -11440,7 +11374,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D130" s="14" t="inlineStr">
+      <c r="D130" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -11465,10 +11399,8 @@
       <c r="J130" s="10" t="n">
         <v>200000</v>
       </c>
-      <c r="K130" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K130" s="10" t="n">
+        <v>459</v>
       </c>
       <c r="L130" s="7" t="inlineStr">
         <is>
@@ -11526,7 +11458,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E131" s="14" t="inlineStr">
+      <c r="E131" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -11687,7 +11619,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E133" s="14" t="inlineStr">
+      <c r="E133" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -11845,7 +11777,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E135" s="14" t="inlineStr">
+      <c r="E135" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -11926,7 +11858,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E136" s="14" t="inlineStr">
+      <c r="E136" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -12000,7 +11932,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D137" s="14" t="inlineStr">
+      <c r="D137" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -12169,7 +12101,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E139" s="14" t="inlineStr">
+      <c r="E139" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -12440,7 +12372,7 @@
       <c r="J142" s="10" t="n">
         <v>150000</v>
       </c>
-      <c r="K142" s="13" t="inlineStr">
+      <c r="K142" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -12656,7 +12588,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D145" s="14" t="inlineStr">
+      <c r="D145" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -12818,12 +12750,12 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D147" s="14" t="inlineStr">
+      <c r="D147" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E147" s="14" t="inlineStr">
+      <c r="E147" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -12902,7 +12834,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E148" s="14" t="inlineStr">
+      <c r="E148" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -13174,7 +13106,7 @@
       <c r="J151" s="10" t="n">
         <v>100000</v>
       </c>
-      <c r="K151" s="13" t="inlineStr">
+      <c r="K151" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -13261,7 +13193,7 @@
       <c r="J152" s="10" t="n">
         <v>50000</v>
       </c>
-      <c r="K152" s="13" t="inlineStr">
+      <c r="K152" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -13394,7 +13326,7 @@
           <t>CFD + Futures</t>
         </is>
       </c>
-      <c r="D154" s="14" t="inlineStr">
+      <c r="D154" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -13423,10 +13355,8 @@
       <c r="J154" s="10" t="n">
         <v>25000</v>
       </c>
-      <c r="K154" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K154" s="10" t="n">
+        <v>189</v>
       </c>
       <c r="L154" s="7" t="inlineStr">
         <is>
@@ -13481,7 +13411,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D155" s="14" t="inlineStr">
+      <c r="D155" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -13506,10 +13436,8 @@
       <c r="J155" s="10" t="n">
         <v>25000</v>
       </c>
-      <c r="K155" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K155" s="10" t="n">
+        <v>189</v>
       </c>
       <c r="L155" s="11" t="inlineStr">
         <is>
@@ -13564,7 +13492,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D156" s="14" t="inlineStr">
+      <c r="D156" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -13589,10 +13517,8 @@
       <c r="J156" s="10" t="n">
         <v>25000</v>
       </c>
-      <c r="K156" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K156" s="10" t="n">
+        <v>189</v>
       </c>
       <c r="L156" s="7" t="inlineStr">
         <is>
@@ -13806,12 +13732,12 @@
       <c r="I2" s="9" t="n">
         <v>325000</v>
       </c>
-      <c r="J2" s="13" t="inlineStr">
+      <c r="J2" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K2" s="13" t="inlineStr">
+      <c r="K2" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -13891,12 +13817,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J3" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="K3" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -13980,12 +13906,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="J4" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K4" s="13" t="inlineStr">
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14042,7 +13968,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -14067,12 +13993,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="K5" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14150,15 +14076,13 @@
       <c r="I6" s="9" t="n">
         <v>1024000</v>
       </c>
-      <c r="J6" s="13" t="inlineStr">
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K6" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K6" s="10" t="n">
+        <v>198</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -14237,12 +14161,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J7" s="13" t="inlineStr">
+      <c r="J7" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K7" s="13" t="inlineStr">
+      <c r="K7" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14322,12 +14246,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J8" s="13" t="inlineStr">
+      <c r="J8" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K8" s="13" t="inlineStr">
+      <c r="K8" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14407,12 +14331,12 @@
       <c r="I9" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="J9" s="13" t="inlineStr">
+      <c r="J9" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K9" s="13" t="inlineStr">
+      <c r="K9" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14475,7 +14399,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -14500,12 +14424,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K10" s="13" t="inlineStr">
+      <c r="K10" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14587,12 +14511,12 @@
       <c r="I11" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K11" s="13" t="inlineStr">
+      <c r="K11" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14672,12 +14596,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J12" s="13" t="inlineStr">
+      <c r="J12" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K12" s="13" t="inlineStr">
+      <c r="K12" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14757,12 +14681,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J13" s="13" t="inlineStr">
+      <c r="J13" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K13" s="13" t="inlineStr">
+      <c r="K13" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14842,12 +14766,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J14" s="13" t="inlineStr">
+      <c r="J14" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K14" s="13" t="inlineStr">
+      <c r="K14" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -14931,12 +14855,12 @@
       <c r="I15" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K15" s="13" t="inlineStr">
+      <c r="K15" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15018,12 +14942,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J16" s="13" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K16" s="13" t="inlineStr">
+      <c r="K16" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15103,12 +15027,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J17" s="13" t="inlineStr">
+      <c r="J17" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K17" s="13" t="inlineStr">
+      <c r="K17" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15188,12 +15112,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J18" s="13" t="inlineStr">
+      <c r="J18" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K18" s="13" t="inlineStr">
+      <c r="K18" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15254,7 +15178,7 @@
           <t>OUI</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -15273,12 +15197,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J19" s="13" t="inlineStr">
+      <c r="J19" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K19" s="13" t="inlineStr">
+      <c r="K19" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15364,15 +15288,13 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K20" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K20" s="10" t="n">
+        <v>58000</v>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
@@ -15455,12 +15377,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
+      <c r="J21" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K21" s="13" t="inlineStr">
+      <c r="K21" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15538,12 +15460,12 @@
       <c r="I22" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="J22" s="13" t="inlineStr">
+      <c r="J22" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K22" s="13" t="inlineStr">
+      <c r="K22" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15623,12 +15545,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J23" s="13" t="inlineStr">
+      <c r="J23" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K23" s="13" t="inlineStr">
+      <c r="K23" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15706,12 +15628,12 @@
       <c r="I24" s="9" t="n">
         <v>400000</v>
       </c>
-      <c r="J24" s="13" t="inlineStr">
+      <c r="J24" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K24" s="13" t="inlineStr">
+      <c r="K24" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15793,15 +15715,13 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="J25" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K25" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K25" s="10" t="n">
+        <v>49</v>
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
@@ -15856,12 +15776,12 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="13" t="inlineStr">
         <is>
           <t>OUI sous conditions</t>
         </is>
@@ -15880,12 +15800,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="J26" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K26" s="13" t="inlineStr">
+      <c r="K26" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -15963,12 +15883,12 @@
       <c r="I27" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="J27" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K27" s="13" t="inlineStr">
+      <c r="K27" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16050,12 +15970,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J28" s="13" t="inlineStr">
+      <c r="J28" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K28" s="13" t="inlineStr">
+      <c r="K28" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16133,15 +16053,13 @@
       <c r="I29" s="12" t="n">
         <v>750000</v>
       </c>
-      <c r="J29" s="13" t="inlineStr">
+      <c r="J29" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K29" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K29" s="10" t="n">
+        <v>2405</v>
       </c>
       <c r="L29" s="11" t="inlineStr">
         <is>
@@ -16222,12 +16140,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J30" s="13" t="inlineStr">
+      <c r="J30" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K30" s="13" t="inlineStr">
+      <c r="K30" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16279,7 +16197,7 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>OUI sur certains comptes</t>
         </is>
@@ -16303,12 +16221,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J31" s="13" t="inlineStr">
+      <c r="J31" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K31" s="13" t="inlineStr">
+      <c r="K31" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16390,12 +16308,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J32" s="13" t="inlineStr">
+      <c r="J32" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K32" s="13" t="inlineStr">
+      <c r="K32" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16479,12 +16397,12 @@
       <c r="I33" s="12" t="n">
         <v>3000000</v>
       </c>
-      <c r="J33" s="13" t="inlineStr">
+      <c r="J33" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K33" s="13" t="inlineStr">
+      <c r="K33" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16564,12 +16482,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J34" s="13" t="inlineStr">
+      <c r="J34" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K34" s="13" t="inlineStr">
+      <c r="K34" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16649,12 +16567,12 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="J35" s="13" t="inlineStr">
+      <c r="J35" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K35" s="13" t="inlineStr">
+      <c r="K35" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16738,12 +16656,12 @@
       <c r="I36" s="9" t="n">
         <v>940000</v>
       </c>
-      <c r="J36" s="13" t="inlineStr">
+      <c r="J36" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K36" s="13" t="inlineStr">
+      <c r="K36" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16821,12 +16739,12 @@
       <c r="I37" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="J37" s="13" t="inlineStr">
+      <c r="J37" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K37" s="13" t="inlineStr">
+      <c r="K37" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
@@ -16910,15 +16828,13 @@
       <c r="I38" s="9" t="n">
         <v>900000</v>
       </c>
-      <c r="J38" s="13" t="inlineStr">
+      <c r="J38" s="14" t="inlineStr">
         <is>
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K38" s="13" t="inlineStr">
-        <is>
-          <t>inconnu</t>
-        </is>
+      <c r="K38" s="10" t="n">
+        <v>1977</v>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ne déduit plus de prix cumulé quand le calcul est inconnu
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpnEpdwNF8V8azepdqLgDD
</commit_message>
<xml_diff>
--- a/docs/prop-firms-capital-max.xlsx
+++ b/docs/prop-firms-capital-max.xlsx
@@ -1218,8 +1218,10 @@
       <c r="J6" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="K6" s="10" t="n">
-        <v>3500</v>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>inconnu</t>
+        </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -15720,8 +15722,10 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K25" s="10" t="n">
-        <v>49</v>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>inconnu</t>
+        </is>
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
@@ -16058,8 +16062,10 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K29" s="10" t="n">
-        <v>2405</v>
+      <c r="K29" s="14" t="inlineStr">
+        <is>
+          <t>inconnu</t>
+        </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
         <is>
@@ -16833,8 +16839,10 @@
           <t>inconnu</t>
         </is>
       </c>
-      <c r="K38" s="10" t="n">
-        <v>1977</v>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>inconnu</t>
+        </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>

</xml_diff>